<commit_message>
Add resonance strength Python and DSL2 C macro
Add Calc_Resonance_Strength.py to compute resonance statistical factor and resonance strength using uncertainties.ufloat, and add Comparison_DSL2_Lexie.C — a ROOT macro for comparing simulated and measured spectra (background fit, Minuit minimization, residuals, and output saving). Update average.C to adjust TPaveText placement and make saved PNG path handling more robust. Also include updated binary spreadsheets Calc_BGT.xlsx and Calc_Width_Lifetime.xlsx.
</commit_message>
<xml_diff>
--- a/Calc_Width_Lifetime.xlsx
+++ b/Calc_Width_Lifetime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{483A74E2-4D99-4AE8-AB2F-7234F7D398BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D197EFE-C280-41F4-95D9-B07525493F30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{54B87DC3-80D2-408F-9ECA-DC6AAEA4FCE2}"/>
+    <workbookView xWindow="348" yWindow="504" windowWidth="12564" windowHeight="12000" xr2:uid="{54B87DC3-80D2-408F-9ECA-DC6AAEA4FCE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
   <si>
     <t>τ (fs)</t>
   </si>
@@ -112,11 +112,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0E+00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,6 +185,13 @@
       <name val="Cambria"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -220,7 +228,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -252,13 +260,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2027,7 +2038,7 @@
         <v>13</v>
       </c>
       <c r="B6" s="6">
-        <v>5.0000000000000001E-3</v>
+        <v>5.8</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>3</v>
@@ -2050,7 +2061,7 @@
       </c>
       <c r="B7" s="3">
         <f>B6/$B$2</f>
-        <v>5.0000000000000001E-9</v>
+        <v>5.7999999999999995E-6</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>8</v>
@@ -2073,7 +2084,7 @@
       </c>
       <c r="B8" s="2">
         <f>B4/$B$6</f>
-        <v>1.3164239138000002E-13</v>
+        <v>1.1348482015517243E-16</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
@@ -2096,7 +2107,7 @@
       </c>
       <c r="B9" s="9">
         <f>B8*$B$3</f>
-        <v>131.64239138000002</v>
+        <v>0.11348482015517243</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>9</v>
@@ -2119,7 +2130,7 @@
       </c>
       <c r="B10" s="8">
         <f>B9*LN(2)</f>
-        <v>91.247552427215865</v>
+        <v>7.8661683126910228E-2</v>
       </c>
       <c r="C10" s="1" t="str">
         <f>C9</f>
@@ -2167,14 +2178,14 @@
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="13">
-        <v>1.1200000000000001</v>
+      <c r="B13" s="14">
+        <v>104000000</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="12">
-        <v>0.18</v>
+      <c r="D13" s="13">
+        <v>3</v>
       </c>
       <c r="F13" s="4">
         <v>1.1000000000000001</v>
@@ -2194,7 +2205,7 @@
       </c>
       <c r="B14" s="2">
         <f>B13/$B$3</f>
-        <v>1.1200000000000001E-15</v>
+        <v>1.04E-7</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>4</v>
@@ -2217,7 +2228,7 @@
       </c>
       <c r="B15" s="7">
         <f>$B$4/B14</f>
-        <v>0.58768924723214289</v>
+        <v>6.3289611240384617E-9</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>3</v>
@@ -2240,7 +2251,7 @@
       </c>
       <c r="B16" s="2">
         <f>B15/$B$2</f>
-        <v>5.8768924723214289E-7</v>
+        <v>6.3289611240384614E-15</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>8</v>
@@ -2263,7 +2274,7 @@
       </c>
       <c r="B17" s="11">
         <f>B13*LN(2)</f>
-        <v>0.77632484222713882</v>
+        <v>72087306.778234303</v>
       </c>
       <c r="C17" s="1" t="str">
         <f>C13</f>
@@ -2271,7 +2282,7 @@
       </c>
       <c r="D17" s="11">
         <f>D13*LN(2)</f>
-        <v>0.12476649250079015</v>
+        <v>2.0794415416798357</v>
       </c>
       <c r="F17" s="4">
         <v>1.5</v>
@@ -2324,7 +2335,16 @@
         <v>0.25346542340893291</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" ht="18.600000000000001">
+      <c r="A21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="10">
+        <v>31.4</v>
+      </c>
+      <c r="D21" s="10">
+        <v>4</v>
+      </c>
       <c r="F21" s="4">
         <v>1.9</v>
       </c>
@@ -2338,6 +2358,17 @@
       </c>
     </row>
     <row r="22" spans="1:8">
+      <c r="A22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="12">
+        <f>B21/LN(2)</f>
+        <v>45.30062428391345</v>
+      </c>
+      <c r="D22" s="12">
+        <f>D21/LN(2)</f>
+        <v>5.7707801635558535</v>
+      </c>
       <c r="F22" s="4">
         <v>2</v>
       </c>

</xml_diff>